<commit_message>
Updated SR and Obs and CodeableConcept
</commit_message>
<xml_diff>
--- a/314e-ig/output/StructureDefinition-observation-lab-nonmicro-314e.xlsx
+++ b/314e-ig/output/StructureDefinition-observation-lab-nonmicro-314e.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3097" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3097" uniqueCount="594">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-19T06:46:39+05:30</t>
+    <t>2026-05-19T11:54:54+05:30</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -715,10 +715,6 @@
     <t>internalIdentifier</t>
   </si>
   <si>
-    <t xml:space="preserve">Identifier
-</t>
-  </si>
-  <si>
     <t>Customer-specific internal identifier whose system SHALL follow the 314e internal naming convention</t>
   </si>
   <si>
@@ -780,7 +776,7 @@
     <t>Observation.identifier.type</t>
   </si>
   <si>
-    <t xml:space="preserve">CodeableConcept
+    <t xml:space="preserve">CodeableConcept {http://314e.com/fhir/ig/StructureDefinition/codeableconcept-314e}
 </t>
   </si>
   <si>
@@ -814,10 +810,14 @@
     <t>Observation.identifier.system</t>
   </si>
   <si>
-    <t>The namespace for the identifier value</t>
-  </si>
-  <si>
-    <t>Establishes the namespace for the value - that is, a URL that describes a set values that are unique.</t>
+    <t>Identifier namespace URI or constrained-format internal identifier-system name</t>
+  </si>
+  <si>
+    <t>Establishes the namespace, issuer, or context in which the identifier value is unique.
+Standard identifiers SHOULD use canonical URIs whenever available.
+For customer-specific or internally defined identifier systems,
+the following naming convention SHALL be used:
+[customer]-[ehr]-[ResourceType]-[resource-subtype]-[eleMent]-[SourceSpecificString]-InternalIdentifier</t>
   </si>
   <si>
     <t>Identifier.system is always case sensitive.</t>
@@ -844,13 +844,15 @@
     <t>Observation.identifier.value</t>
   </si>
   <si>
-    <t>The value that is unique</t>
-  </si>
-  <si>
-    <t>The portion of the identifier typically relevant to the user and which is unique within the context of the system.</t>
-  </si>
-  <si>
-    <t>If the value is a full URI, then the system SHALL be urn:ietf:rfc:3986.  The value's primary purpose is computational mapping.  As a result, it may be normalized for comparison purposes (e.g. removing non-significant whitespace, dashes, etc.)  A value formatted for human display can be conveyed using the [Rendered Value extension](http://hl7.org/fhir/R4/extension-rendered-value.html). Identifier.value is to be treated as case sensitive unless knowledge of the Identifier.system allows the processer to be confident that non-case-sensitive processing is safe.</t>
+    <t>The identifier value</t>
+  </si>
+  <si>
+    <t>The portion of the identifier typically relevant to the user
+and which is unique within the context of the system.</t>
+  </si>
+  <si>
+    <t>If Identifier.value is populated,
+Identifier.system SHALL also be populated.</t>
   </si>
   <si>
     <t>123456</t>
@@ -871,7 +873,7 @@
     <t>Observation.identifier.period</t>
   </si>
   <si>
-    <t xml:space="preserve">Period
+    <t xml:space="preserve">Period {http://314e.com/fhir/ig/StructureDefinition/period-314e}
 </t>
   </si>
   <si>
@@ -1016,10 +1018,6 @@
   </si>
   <si>
     <t>2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CodeableConcept {http://314e.com/fhir/ig/StructureDefinition/codeableconcept-314e}
-</t>
   </si>
   <si>
     <t>(QI) Classification of  type of observation</t>
@@ -1347,6 +1345,10 @@
   </si>
   <si>
     <t>Observation.dataAbsentReason</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CodeableConcept
+</t>
   </si>
   <si>
     <t>Why the result is missing</t>
@@ -4693,13 +4695,13 @@
         <v>93</v>
       </c>
       <c r="K21" t="s" s="2">
+        <v>208</v>
+      </c>
+      <c r="L21" t="s" s="2">
         <v>219</v>
       </c>
-      <c r="L21" t="s" s="2">
+      <c r="M21" t="s" s="2">
         <v>220</v>
-      </c>
-      <c r="M21" t="s" s="2">
-        <v>221</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" t="s" s="2">
@@ -4787,10 +4789,10 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
+        <v>221</v>
+      </c>
+      <c r="B22" t="s" s="2">
         <v>222</v>
-      </c>
-      <c r="B22" t="s" s="2">
-        <v>223</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -4905,10 +4907,10 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
+        <v>223</v>
+      </c>
+      <c r="B23" t="s" s="2">
         <v>224</v>
-      </c>
-      <c r="B23" t="s" s="2">
-        <v>225</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -5025,10 +5027,10 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
+        <v>225</v>
+      </c>
+      <c r="B24" t="s" s="2">
         <v>226</v>
-      </c>
-      <c r="B24" t="s" s="2">
-        <v>227</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -5054,16 +5056,16 @@
         <v>168</v>
       </c>
       <c r="L24" t="s" s="2">
+        <v>227</v>
+      </c>
+      <c r="M24" t="s" s="2">
         <v>228</v>
       </c>
-      <c r="M24" t="s" s="2">
+      <c r="N24" t="s" s="2">
         <v>229</v>
       </c>
-      <c r="N24" t="s" s="2">
+      <c r="O24" t="s" s="2">
         <v>230</v>
-      </c>
-      <c r="O24" t="s" s="2">
-        <v>231</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>20</v>
@@ -5088,31 +5090,31 @@
         <v>20</v>
       </c>
       <c r="X24" t="s" s="2">
+        <v>231</v>
+      </c>
+      <c r="Y24" t="s" s="2">
         <v>232</v>
       </c>
-      <c r="Y24" t="s" s="2">
+      <c r="Z24" t="s" s="2">
         <v>233</v>
       </c>
-      <c r="Z24" t="s" s="2">
+      <c r="AA24" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AB24" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AC24" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AD24" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AE24" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AF24" t="s" s="2">
         <v>234</v>
-      </c>
-      <c r="AA24" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AB24" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AC24" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AD24" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AE24" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AF24" t="s" s="2">
-        <v>235</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>80</v>
@@ -5136,7 +5138,7 @@
         <v>191</v>
       </c>
       <c r="AN24" t="s" s="2">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AO24" t="s" s="2">
         <v>20</v>
@@ -5147,10 +5149,10 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
+        <v>236</v>
+      </c>
+      <c r="B25" t="s" s="2">
         <v>237</v>
-      </c>
-      <c r="B25" t="s" s="2">
-        <v>238</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -5173,19 +5175,19 @@
         <v>93</v>
       </c>
       <c r="K25" t="s" s="2">
+        <v>238</v>
+      </c>
+      <c r="L25" t="s" s="2">
         <v>239</v>
       </c>
-      <c r="L25" t="s" s="2">
+      <c r="M25" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="M25" t="s" s="2">
+      <c r="N25" t="s" s="2">
         <v>241</v>
       </c>
-      <c r="N25" t="s" s="2">
+      <c r="O25" t="s" s="2">
         <v>242</v>
-      </c>
-      <c r="O25" t="s" s="2">
-        <v>243</v>
       </c>
       <c r="P25" t="s" s="2">
         <v>20</v>
@@ -5213,28 +5215,28 @@
         <v>150</v>
       </c>
       <c r="Y25" t="s" s="2">
+        <v>243</v>
+      </c>
+      <c r="Z25" t="s" s="2">
         <v>244</v>
       </c>
-      <c r="Z25" t="s" s="2">
+      <c r="AA25" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AB25" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AC25" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AD25" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AE25" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AF25" t="s" s="2">
         <v>245</v>
-      </c>
-      <c r="AA25" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AB25" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AC25" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AD25" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AE25" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AF25" t="s" s="2">
-        <v>246</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>80</v>
@@ -5255,10 +5257,10 @@
         <v>20</v>
       </c>
       <c r="AM25" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="AN25" t="s" s="2">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AO25" t="s" s="2">
         <v>20</v>
@@ -5269,10 +5271,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
+        <v>247</v>
+      </c>
+      <c r="B26" t="s" s="2">
         <v>248</v>
-      </c>
-      <c r="B26" t="s" s="2">
-        <v>249</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -5298,16 +5300,16 @@
         <v>134</v>
       </c>
       <c r="L26" t="s" s="2">
+        <v>249</v>
+      </c>
+      <c r="M26" t="s" s="2">
         <v>250</v>
       </c>
-      <c r="M26" t="s" s="2">
+      <c r="N26" t="s" s="2">
         <v>251</v>
       </c>
-      <c r="N26" t="s" s="2">
+      <c r="O26" t="s" s="2">
         <v>252</v>
-      </c>
-      <c r="O26" t="s" s="2">
-        <v>253</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>20</v>
@@ -5320,43 +5322,43 @@
         <v>20</v>
       </c>
       <c r="T26" t="s" s="2">
+        <v>253</v>
+      </c>
+      <c r="U26" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="V26" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="W26" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="X26" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Y26" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Z26" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AA26" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AB26" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AC26" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AD26" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AE26" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AF26" t="s" s="2">
         <v>254</v>
-      </c>
-      <c r="U26" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="V26" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="W26" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="X26" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Y26" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Z26" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AA26" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AB26" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AC26" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AD26" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AE26" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AF26" t="s" s="2">
-        <v>255</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>80</v>
@@ -5377,10 +5379,10 @@
         <v>20</v>
       </c>
       <c r="AM26" t="s" s="2">
+        <v>255</v>
+      </c>
+      <c r="AN26" t="s" s="2">
         <v>256</v>
-      </c>
-      <c r="AN26" t="s" s="2">
-        <v>257</v>
       </c>
       <c r="AO26" t="s" s="2">
         <v>20</v>
@@ -5391,10 +5393,10 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
+        <v>257</v>
+      </c>
+      <c r="B27" t="s" s="2">
         <v>258</v>
-      </c>
-      <c r="B27" t="s" s="2">
-        <v>259</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -5420,13 +5422,13 @@
         <v>106</v>
       </c>
       <c r="L27" t="s" s="2">
+        <v>259</v>
+      </c>
+      <c r="M27" t="s" s="2">
         <v>260</v>
       </c>
-      <c r="M27" t="s" s="2">
+      <c r="N27" t="s" s="2">
         <v>261</v>
-      </c>
-      <c r="N27" t="s" s="2">
-        <v>262</v>
       </c>
       <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
@@ -5440,43 +5442,43 @@
         <v>20</v>
       </c>
       <c r="T27" t="s" s="2">
+        <v>262</v>
+      </c>
+      <c r="U27" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="V27" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="W27" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="X27" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Y27" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Z27" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AA27" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AB27" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AC27" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AD27" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AE27" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AF27" t="s" s="2">
         <v>263</v>
-      </c>
-      <c r="U27" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="V27" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="W27" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="X27" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Y27" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Z27" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AA27" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AB27" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AC27" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AD27" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AE27" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AF27" t="s" s="2">
-        <v>264</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>80</v>
@@ -5497,10 +5499,10 @@
         <v>20</v>
       </c>
       <c r="AM27" t="s" s="2">
+        <v>264</v>
+      </c>
+      <c r="AN27" t="s" s="2">
         <v>265</v>
-      </c>
-      <c r="AN27" t="s" s="2">
-        <v>266</v>
       </c>
       <c r="AO27" t="s" s="2">
         <v>20</v>
@@ -5511,10 +5513,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
+        <v>266</v>
+      </c>
+      <c r="B28" t="s" s="2">
         <v>267</v>
-      </c>
-      <c r="B28" t="s" s="2">
-        <v>268</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -5537,13 +5539,13 @@
         <v>93</v>
       </c>
       <c r="K28" t="s" s="2">
+        <v>268</v>
+      </c>
+      <c r="L28" t="s" s="2">
         <v>269</v>
       </c>
-      <c r="L28" t="s" s="2">
+      <c r="M28" t="s" s="2">
         <v>270</v>
-      </c>
-      <c r="M28" t="s" s="2">
-        <v>271</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -5594,7 +5596,7 @@
         <v>20</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>80</v>
@@ -5615,10 +5617,10 @@
         <v>20</v>
       </c>
       <c r="AM28" t="s" s="2">
+        <v>272</v>
+      </c>
+      <c r="AN28" t="s" s="2">
         <v>273</v>
-      </c>
-      <c r="AN28" t="s" s="2">
-        <v>274</v>
       </c>
       <c r="AO28" t="s" s="2">
         <v>20</v>
@@ -5629,10 +5631,10 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
+        <v>274</v>
+      </c>
+      <c r="B29" t="s" s="2">
         <v>275</v>
-      </c>
-      <c r="B29" t="s" s="2">
-        <v>276</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -5655,16 +5657,16 @@
         <v>93</v>
       </c>
       <c r="K29" t="s" s="2">
+        <v>276</v>
+      </c>
+      <c r="L29" t="s" s="2">
         <v>277</v>
       </c>
-      <c r="L29" t="s" s="2">
+      <c r="M29" t="s" s="2">
         <v>278</v>
       </c>
-      <c r="M29" t="s" s="2">
+      <c r="N29" t="s" s="2">
         <v>279</v>
-      </c>
-      <c r="N29" t="s" s="2">
-        <v>280</v>
       </c>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
@@ -5714,7 +5716,7 @@
         <v>20</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>80</v>
@@ -5735,10 +5737,10 @@
         <v>20</v>
       </c>
       <c r="AM29" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="AN29" t="s" s="2">
         <v>282</v>
-      </c>
-      <c r="AN29" t="s" s="2">
-        <v>283</v>
       </c>
       <c r="AO29" t="s" s="2">
         <v>20</v>
@@ -5749,14 +5751,14 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
@@ -5775,17 +5777,17 @@
         <v>93</v>
       </c>
       <c r="K30" t="s" s="2">
+        <v>285</v>
+      </c>
+      <c r="L30" t="s" s="2">
         <v>286</v>
       </c>
-      <c r="L30" t="s" s="2">
+      <c r="M30" t="s" s="2">
         <v>287</v>
-      </c>
-      <c r="M30" t="s" s="2">
-        <v>288</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" t="s" s="2">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="P30" t="s" s="2">
         <v>20</v>
@@ -5834,7 +5836,7 @@
         <v>20</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>80</v>
@@ -5849,16 +5851,16 @@
         <v>104</v>
       </c>
       <c r="AK30" t="s" s="2">
+        <v>289</v>
+      </c>
+      <c r="AL30" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AM30" t="s" s="2">
         <v>290</v>
       </c>
-      <c r="AL30" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AM30" t="s" s="2">
+      <c r="AN30" t="s" s="2">
         <v>291</v>
-      </c>
-      <c r="AN30" t="s" s="2">
-        <v>292</v>
       </c>
       <c r="AO30" t="s" s="2">
         <v>20</v>
@@ -5869,14 +5871,14 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
@@ -5895,16 +5897,16 @@
         <v>93</v>
       </c>
       <c r="K31" t="s" s="2">
+        <v>294</v>
+      </c>
+      <c r="L31" t="s" s="2">
         <v>295</v>
       </c>
-      <c r="L31" t="s" s="2">
+      <c r="M31" t="s" s="2">
         <v>296</v>
       </c>
-      <c r="M31" t="s" s="2">
+      <c r="N31" t="s" s="2">
         <v>297</v>
-      </c>
-      <c r="N31" t="s" s="2">
-        <v>298</v>
       </c>
       <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
@@ -5954,7 +5956,7 @@
         <v>20</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>80</v>
@@ -5969,16 +5971,16 @@
         <v>104</v>
       </c>
       <c r="AK31" t="s" s="2">
+        <v>298</v>
+      </c>
+      <c r="AL31" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AM31" t="s" s="2">
         <v>299</v>
       </c>
-      <c r="AL31" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AM31" t="s" s="2">
+      <c r="AN31" t="s" s="2">
         <v>300</v>
-      </c>
-      <c r="AN31" t="s" s="2">
-        <v>301</v>
       </c>
       <c r="AO31" t="s" s="2">
         <v>20</v>
@@ -5989,10 +5991,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -6018,16 +6020,16 @@
         <v>168</v>
       </c>
       <c r="L32" t="s" s="2">
+        <v>302</v>
+      </c>
+      <c r="M32" t="s" s="2">
         <v>303</v>
       </c>
-      <c r="M32" t="s" s="2">
+      <c r="N32" t="s" s="2">
         <v>304</v>
       </c>
-      <c r="N32" t="s" s="2">
+      <c r="O32" t="s" s="2">
         <v>305</v>
-      </c>
-      <c r="O32" t="s" s="2">
-        <v>306</v>
       </c>
       <c r="P32" t="s" s="2">
         <v>20</v>
@@ -6052,14 +6054,14 @@
         <v>20</v>
       </c>
       <c r="X32" t="s" s="2">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="Y32" t="s" s="2">
+        <v>306</v>
+      </c>
+      <c r="Z32" t="s" s="2">
         <v>307</v>
       </c>
-      <c r="Z32" t="s" s="2">
-        <v>308</v>
-      </c>
       <c r="AA32" t="s" s="2">
         <v>20</v>
       </c>
@@ -6076,7 +6078,7 @@
         <v>20</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>92</v>
@@ -6091,19 +6093,19 @@
         <v>104</v>
       </c>
       <c r="AK32" t="s" s="2">
+        <v>308</v>
+      </c>
+      <c r="AL32" t="s" s="2">
         <v>309</v>
       </c>
-      <c r="AL32" t="s" s="2">
+      <c r="AM32" t="s" s="2">
         <v>310</v>
       </c>
-      <c r="AM32" t="s" s="2">
+      <c r="AN32" t="s" s="2">
         <v>311</v>
       </c>
-      <c r="AN32" t="s" s="2">
+      <c r="AO32" t="s" s="2">
         <v>312</v>
-      </c>
-      <c r="AO32" t="s" s="2">
-        <v>313</v>
       </c>
       <c r="AP32" t="s" s="2">
         <v>20</v>
@@ -6111,10 +6113,10 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -6122,7 +6124,7 @@
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="G33" t="s" s="2">
         <v>81</v>
@@ -6137,19 +6139,19 @@
         <v>20</v>
       </c>
       <c r="K33" t="s" s="2">
+        <v>238</v>
+      </c>
+      <c r="L33" t="s" s="2">
+        <v>315</v>
+      </c>
+      <c r="M33" t="s" s="2">
         <v>316</v>
       </c>
-      <c r="L33" t="s" s="2">
+      <c r="N33" t="s" s="2">
         <v>317</v>
       </c>
-      <c r="M33" t="s" s="2">
+      <c r="O33" t="s" s="2">
         <v>318</v>
-      </c>
-      <c r="N33" t="s" s="2">
-        <v>319</v>
-      </c>
-      <c r="O33" t="s" s="2">
-        <v>320</v>
       </c>
       <c r="P33" t="s" s="2">
         <v>20</v>
@@ -6177,10 +6179,10 @@
         <v>172</v>
       </c>
       <c r="Y33" t="s" s="2">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="Z33" t="s" s="2">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="AA33" t="s" s="2">
         <v>20</v>
@@ -6196,7 +6198,7 @@
         <v>119</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>80</v>
@@ -6220,10 +6222,10 @@
         <v>20</v>
       </c>
       <c r="AN33" t="s" s="2">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="AO33" t="s" s="2">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="AP33" t="s" s="2">
         <v>20</v>
@@ -6231,13 +6233,13 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C34" t="s" s="2">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D34" t="s" s="2">
         <v>20</v>
@@ -6259,19 +6261,19 @@
         <v>20</v>
       </c>
       <c r="K34" t="s" s="2">
+        <v>238</v>
+      </c>
+      <c r="L34" t="s" s="2">
+        <v>315</v>
+      </c>
+      <c r="M34" t="s" s="2">
         <v>316</v>
       </c>
-      <c r="L34" t="s" s="2">
+      <c r="N34" t="s" s="2">
         <v>317</v>
       </c>
-      <c r="M34" t="s" s="2">
+      <c r="O34" t="s" s="2">
         <v>318</v>
-      </c>
-      <c r="N34" t="s" s="2">
-        <v>319</v>
-      </c>
-      <c r="O34" t="s" s="2">
-        <v>320</v>
       </c>
       <c r="P34" t="s" s="2">
         <v>20</v>
@@ -6281,29 +6283,29 @@
         <v>20</v>
       </c>
       <c r="S34" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="T34" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="U34" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="V34" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="W34" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="X34" t="s" s="2">
+        <v>231</v>
+      </c>
+      <c r="Y34" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="Z34" t="s" s="2">
         <v>327</v>
       </c>
-      <c r="T34" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="U34" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="V34" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="W34" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="X34" t="s" s="2">
-        <v>232</v>
-      </c>
-      <c r="Y34" t="s" s="2">
-        <v>328</v>
-      </c>
-      <c r="Z34" t="s" s="2">
-        <v>329</v>
-      </c>
       <c r="AA34" t="s" s="2">
         <v>20</v>
       </c>
@@ -6320,7 +6322,7 @@
         <v>20</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>80</v>
@@ -6344,10 +6346,10 @@
         <v>20</v>
       </c>
       <c r="AN34" t="s" s="2">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="AO34" t="s" s="2">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="AP34" t="s" s="2">
         <v>20</v>
@@ -6355,13 +6357,13 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C35" t="s" s="2">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D35" t="s" s="2">
         <v>20</v>
@@ -6383,19 +6385,19 @@
         <v>20</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="O35" t="s" s="2">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="P35" t="s" s="2">
         <v>20</v>
@@ -6420,11 +6422,11 @@
         <v>20</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="Y35" s="2"/>
       <c r="Z35" t="s" s="2">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="AA35" t="s" s="2">
         <v>20</v>
@@ -6442,7 +6444,7 @@
         <v>20</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>80</v>
@@ -6466,10 +6468,10 @@
         <v>20</v>
       </c>
       <c r="AN35" t="s" s="2">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="AO35" t="s" s="2">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="AP35" t="s" s="2">
         <v>20</v>
@@ -6477,14 +6479,14 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" t="s" s="2">
@@ -6503,19 +6505,19 @@
         <v>93</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>316</v>
+        <v>238</v>
       </c>
       <c r="L36" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="M36" t="s" s="2">
+        <v>336</v>
+      </c>
+      <c r="N36" t="s" s="2">
         <v>337</v>
       </c>
-      <c r="M36" t="s" s="2">
+      <c r="O36" t="s" s="2">
         <v>338</v>
-      </c>
-      <c r="N36" t="s" s="2">
-        <v>339</v>
-      </c>
-      <c r="O36" t="s" s="2">
-        <v>340</v>
       </c>
       <c r="P36" t="s" s="2">
         <v>20</v>
@@ -6543,10 +6545,10 @@
         <v>150</v>
       </c>
       <c r="Y36" t="s" s="2">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="Z36" t="s" s="2">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="AA36" t="s" s="2">
         <v>20</v>
@@ -6564,7 +6566,7 @@
         <v>20</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>92</v>
@@ -6579,30 +6581,30 @@
         <v>104</v>
       </c>
       <c r="AK36" t="s" s="2">
+        <v>341</v>
+      </c>
+      <c r="AL36" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="AM36" t="s" s="2">
         <v>343</v>
       </c>
-      <c r="AL36" t="s" s="2">
+      <c r="AN36" t="s" s="2">
         <v>344</v>
       </c>
-      <c r="AM36" t="s" s="2">
+      <c r="AO36" t="s" s="2">
         <v>345</v>
       </c>
-      <c r="AN36" t="s" s="2">
+      <c r="AP36" t="s" s="2">
         <v>346</v>
-      </c>
-      <c r="AO36" t="s" s="2">
-        <v>347</v>
-      </c>
-      <c r="AP36" t="s" s="2">
-        <v>348</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -6625,19 +6627,19 @@
         <v>93</v>
       </c>
       <c r="K37" t="s" s="2">
+        <v>348</v>
+      </c>
+      <c r="L37" t="s" s="2">
+        <v>349</v>
+      </c>
+      <c r="M37" t="s" s="2">
         <v>350</v>
       </c>
-      <c r="L37" t="s" s="2">
+      <c r="N37" t="s" s="2">
         <v>351</v>
       </c>
-      <c r="M37" t="s" s="2">
+      <c r="O37" t="s" s="2">
         <v>352</v>
-      </c>
-      <c r="N37" t="s" s="2">
-        <v>353</v>
-      </c>
-      <c r="O37" t="s" s="2">
-        <v>354</v>
       </c>
       <c r="P37" t="s" s="2">
         <v>20</v>
@@ -6686,7 +6688,7 @@
         <v>20</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>80</v>
@@ -6701,19 +6703,19 @@
         <v>104</v>
       </c>
       <c r="AK37" t="s" s="2">
+        <v>353</v>
+      </c>
+      <c r="AL37" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AM37" t="s" s="2">
+        <v>354</v>
+      </c>
+      <c r="AN37" t="s" s="2">
         <v>355</v>
       </c>
-      <c r="AL37" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AM37" t="s" s="2">
+      <c r="AO37" t="s" s="2">
         <v>356</v>
-      </c>
-      <c r="AN37" t="s" s="2">
-        <v>357</v>
-      </c>
-      <c r="AO37" t="s" s="2">
-        <v>358</v>
       </c>
       <c r="AP37" t="s" s="2">
         <v>20</v>
@@ -6721,10 +6723,10 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -6747,16 +6749,16 @@
         <v>93</v>
       </c>
       <c r="K38" t="s" s="2">
+        <v>358</v>
+      </c>
+      <c r="L38" t="s" s="2">
+        <v>359</v>
+      </c>
+      <c r="M38" t="s" s="2">
         <v>360</v>
       </c>
-      <c r="L38" t="s" s="2">
+      <c r="N38" t="s" s="2">
         <v>361</v>
-      </c>
-      <c r="M38" t="s" s="2">
-        <v>362</v>
-      </c>
-      <c r="N38" t="s" s="2">
-        <v>363</v>
       </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
@@ -6806,7 +6808,7 @@
         <v>20</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>80</v>
@@ -6827,13 +6829,13 @@
         <v>20</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AN38" t="s" s="2">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="AO38" t="s" s="2">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="AP38" t="s" s="2">
         <v>20</v>
@@ -6841,14 +6843,14 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" t="s" s="2">
@@ -6867,19 +6869,19 @@
         <v>93</v>
       </c>
       <c r="K39" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="L39" t="s" s="2">
+        <v>366</v>
+      </c>
+      <c r="M39" t="s" s="2">
         <v>367</v>
       </c>
-      <c r="L39" t="s" s="2">
+      <c r="N39" t="s" s="2">
         <v>368</v>
       </c>
-      <c r="M39" t="s" s="2">
+      <c r="O39" t="s" s="2">
         <v>369</v>
-      </c>
-      <c r="N39" t="s" s="2">
-        <v>370</v>
-      </c>
-      <c r="O39" t="s" s="2">
-        <v>371</v>
       </c>
       <c r="P39" t="s" s="2">
         <v>20</v>
@@ -6928,7 +6930,7 @@
         <v>20</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>80</v>
@@ -6943,19 +6945,19 @@
         <v>104</v>
       </c>
       <c r="AK39" t="s" s="2">
+        <v>370</v>
+      </c>
+      <c r="AL39" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AM39" t="s" s="2">
+        <v>371</v>
+      </c>
+      <c r="AN39" t="s" s="2">
         <v>372</v>
       </c>
-      <c r="AL39" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AM39" t="s" s="2">
+      <c r="AO39" t="s" s="2">
         <v>373</v>
-      </c>
-      <c r="AN39" t="s" s="2">
-        <v>374</v>
-      </c>
-      <c r="AO39" t="s" s="2">
-        <v>375</v>
       </c>
       <c r="AP39" t="s" s="2">
         <v>20</v>
@@ -6963,14 +6965,14 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="E40" s="2"/>
       <c r="F40" t="s" s="2">
@@ -6989,19 +6991,19 @@
         <v>93</v>
       </c>
       <c r="K40" t="s" s="2">
+        <v>376</v>
+      </c>
+      <c r="L40" t="s" s="2">
+        <v>377</v>
+      </c>
+      <c r="M40" t="s" s="2">
         <v>378</v>
       </c>
-      <c r="L40" t="s" s="2">
+      <c r="N40" t="s" s="2">
         <v>379</v>
       </c>
-      <c r="M40" t="s" s="2">
+      <c r="O40" t="s" s="2">
         <v>380</v>
-      </c>
-      <c r="N40" t="s" s="2">
-        <v>381</v>
-      </c>
-      <c r="O40" t="s" s="2">
-        <v>382</v>
       </c>
       <c r="P40" t="s" s="2">
         <v>20</v>
@@ -7050,7 +7052,7 @@
         <v>20</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>80</v>
@@ -7059,25 +7061,25 @@
         <v>92</v>
       </c>
       <c r="AI40" t="s" s="2">
+        <v>381</v>
+      </c>
+      <c r="AJ40" t="s" s="2">
+        <v>382</v>
+      </c>
+      <c r="AK40" t="s" s="2">
         <v>383</v>
       </c>
-      <c r="AJ40" t="s" s="2">
+      <c r="AL40" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AM40" t="s" s="2">
         <v>384</v>
       </c>
-      <c r="AK40" t="s" s="2">
+      <c r="AN40" t="s" s="2">
         <v>385</v>
       </c>
-      <c r="AL40" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AM40" t="s" s="2">
+      <c r="AO40" t="s" s="2">
         <v>386</v>
-      </c>
-      <c r="AN40" t="s" s="2">
-        <v>387</v>
-      </c>
-      <c r="AO40" t="s" s="2">
-        <v>388</v>
       </c>
       <c r="AP40" t="s" s="2">
         <v>20</v>
@@ -7085,10 +7087,10 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -7111,16 +7113,16 @@
         <v>93</v>
       </c>
       <c r="K41" t="s" s="2">
+        <v>388</v>
+      </c>
+      <c r="L41" t="s" s="2">
+        <v>389</v>
+      </c>
+      <c r="M41" t="s" s="2">
         <v>390</v>
       </c>
-      <c r="L41" t="s" s="2">
+      <c r="N41" t="s" s="2">
         <v>391</v>
-      </c>
-      <c r="M41" t="s" s="2">
-        <v>392</v>
-      </c>
-      <c r="N41" t="s" s="2">
-        <v>393</v>
       </c>
       <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
@@ -7170,7 +7172,7 @@
         <v>20</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>80</v>
@@ -7191,13 +7193,13 @@
         <v>20</v>
       </c>
       <c r="AM41" t="s" s="2">
+        <v>392</v>
+      </c>
+      <c r="AN41" t="s" s="2">
+        <v>393</v>
+      </c>
+      <c r="AO41" t="s" s="2">
         <v>394</v>
-      </c>
-      <c r="AN41" t="s" s="2">
-        <v>395</v>
-      </c>
-      <c r="AO41" t="s" s="2">
-        <v>396</v>
       </c>
       <c r="AP41" t="s" s="2">
         <v>20</v>
@@ -7205,10 +7207,10 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -7231,17 +7233,17 @@
         <v>93</v>
       </c>
       <c r="K42" t="s" s="2">
+        <v>396</v>
+      </c>
+      <c r="L42" t="s" s="2">
+        <v>397</v>
+      </c>
+      <c r="M42" t="s" s="2">
         <v>398</v>
-      </c>
-      <c r="L42" t="s" s="2">
-        <v>399</v>
-      </c>
-      <c r="M42" t="s" s="2">
-        <v>400</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" t="s" s="2">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="P42" t="s" s="2">
         <v>20</v>
@@ -7290,7 +7292,7 @@
         <v>20</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>80</v>
@@ -7305,19 +7307,19 @@
         <v>104</v>
       </c>
       <c r="AK42" t="s" s="2">
+        <v>400</v>
+      </c>
+      <c r="AL42" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AM42" t="s" s="2">
+        <v>401</v>
+      </c>
+      <c r="AN42" t="s" s="2">
         <v>402</v>
       </c>
-      <c r="AL42" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AM42" t="s" s="2">
+      <c r="AO42" t="s" s="2">
         <v>403</v>
-      </c>
-      <c r="AN42" t="s" s="2">
-        <v>404</v>
-      </c>
-      <c r="AO42" t="s" s="2">
-        <v>405</v>
       </c>
       <c r="AP42" t="s" s="2">
         <v>20</v>
@@ -7325,10 +7327,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -7351,19 +7353,19 @@
         <v>93</v>
       </c>
       <c r="K43" t="s" s="2">
+        <v>405</v>
+      </c>
+      <c r="L43" t="s" s="2">
+        <v>406</v>
+      </c>
+      <c r="M43" t="s" s="2">
         <v>407</v>
       </c>
-      <c r="L43" t="s" s="2">
+      <c r="N43" t="s" s="2">
         <v>408</v>
       </c>
-      <c r="M43" t="s" s="2">
+      <c r="O43" t="s" s="2">
         <v>409</v>
-      </c>
-      <c r="N43" t="s" s="2">
-        <v>410</v>
-      </c>
-      <c r="O43" t="s" s="2">
-        <v>411</v>
       </c>
       <c r="P43" t="s" s="2">
         <v>20</v>
@@ -7412,7 +7414,7 @@
         <v>20</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>80</v>
@@ -7421,36 +7423,36 @@
         <v>92</v>
       </c>
       <c r="AI43" t="s" s="2">
+        <v>410</v>
+      </c>
+      <c r="AJ43" t="s" s="2">
+        <v>411</v>
+      </c>
+      <c r="AK43" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AL43" t="s" s="2">
         <v>412</v>
       </c>
-      <c r="AJ43" t="s" s="2">
+      <c r="AM43" t="s" s="2">
         <v>413</v>
       </c>
-      <c r="AK43" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AL43" t="s" s="2">
+      <c r="AN43" t="s" s="2">
         <v>414</v>
       </c>
-      <c r="AM43" t="s" s="2">
+      <c r="AO43" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AP43" t="s" s="2">
         <v>415</v>
-      </c>
-      <c r="AN43" t="s" s="2">
-        <v>416</v>
-      </c>
-      <c r="AO43" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AP43" t="s" s="2">
-        <v>417</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -7473,19 +7475,19 @@
         <v>20</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>239</v>
+        <v>417</v>
       </c>
       <c r="L44" t="s" s="2">
+        <v>418</v>
+      </c>
+      <c r="M44" t="s" s="2">
         <v>419</v>
       </c>
-      <c r="M44" t="s" s="2">
+      <c r="N44" t="s" s="2">
         <v>420</v>
       </c>
-      <c r="N44" t="s" s="2">
+      <c r="O44" t="s" s="2">
         <v>421</v>
-      </c>
-      <c r="O44" t="s" s="2">
-        <v>422</v>
       </c>
       <c r="P44" t="s" s="2">
         <v>20</v>
@@ -7513,11 +7515,11 @@
         <v>150</v>
       </c>
       <c r="Y44" t="s" s="2">
+        <v>422</v>
+      </c>
+      <c r="Z44" t="s" s="2">
         <v>423</v>
       </c>
-      <c r="Z44" t="s" s="2">
-        <v>424</v>
-      </c>
       <c r="AA44" t="s" s="2">
         <v>20</v>
       </c>
@@ -7534,7 +7536,7 @@
         <v>20</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>80</v>
@@ -7543,7 +7545,7 @@
         <v>92</v>
       </c>
       <c r="AI44" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="AJ44" t="s" s="2">
         <v>104</v>
@@ -7558,7 +7560,7 @@
         <v>191</v>
       </c>
       <c r="AN44" t="s" s="2">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="AO44" t="s" s="2">
         <v>20</v>
@@ -7569,14 +7571,14 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
@@ -7595,19 +7597,19 @@
         <v>20</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>316</v>
+        <v>238</v>
       </c>
       <c r="L45" t="s" s="2">
+        <v>428</v>
+      </c>
+      <c r="M45" t="s" s="2">
         <v>429</v>
       </c>
-      <c r="M45" t="s" s="2">
+      <c r="N45" t="s" s="2">
         <v>430</v>
       </c>
-      <c r="N45" t="s" s="2">
+      <c r="O45" t="s" s="2">
         <v>431</v>
-      </c>
-      <c r="O45" t="s" s="2">
-        <v>432</v>
       </c>
       <c r="P45" t="s" s="2">
         <v>20</v>
@@ -7635,11 +7637,11 @@
         <v>150</v>
       </c>
       <c r="Y45" t="s" s="2">
+        <v>432</v>
+      </c>
+      <c r="Z45" t="s" s="2">
         <v>433</v>
       </c>
-      <c r="Z45" t="s" s="2">
-        <v>434</v>
-      </c>
       <c r="AA45" t="s" s="2">
         <v>20</v>
       </c>
@@ -7656,7 +7658,7 @@
         <v>20</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>80</v>
@@ -7674,27 +7676,27 @@
         <v>20</v>
       </c>
       <c r="AL45" t="s" s="2">
+        <v>434</v>
+      </c>
+      <c r="AM45" t="s" s="2">
         <v>435</v>
       </c>
-      <c r="AM45" t="s" s="2">
+      <c r="AN45" t="s" s="2">
         <v>436</v>
       </c>
-      <c r="AN45" t="s" s="2">
+      <c r="AO45" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AP45" t="s" s="2">
         <v>437</v>
-      </c>
-      <c r="AO45" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AP45" t="s" s="2">
-        <v>438</v>
       </c>
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -7717,19 +7719,19 @@
         <v>20</v>
       </c>
       <c r="K46" t="s" s="2">
+        <v>439</v>
+      </c>
+      <c r="L46" t="s" s="2">
         <v>440</v>
       </c>
-      <c r="L46" t="s" s="2">
+      <c r="M46" t="s" s="2">
         <v>441</v>
       </c>
-      <c r="M46" t="s" s="2">
+      <c r="N46" t="s" s="2">
         <v>442</v>
       </c>
-      <c r="N46" t="s" s="2">
+      <c r="O46" t="s" s="2">
         <v>443</v>
-      </c>
-      <c r="O46" t="s" s="2">
-        <v>444</v>
       </c>
       <c r="P46" t="s" s="2">
         <v>20</v>
@@ -7778,7 +7780,7 @@
         <v>20</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>80</v>
@@ -7799,10 +7801,10 @@
         <v>20</v>
       </c>
       <c r="AM46" t="s" s="2">
+        <v>444</v>
+      </c>
+      <c r="AN46" t="s" s="2">
         <v>445</v>
-      </c>
-      <c r="AN46" t="s" s="2">
-        <v>446</v>
       </c>
       <c r="AO46" t="s" s="2">
         <v>20</v>
@@ -7813,10 +7815,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7839,16 +7841,16 @@
         <v>20</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>316</v>
+        <v>238</v>
       </c>
       <c r="L47" t="s" s="2">
+        <v>447</v>
+      </c>
+      <c r="M47" t="s" s="2">
         <v>448</v>
       </c>
-      <c r="M47" t="s" s="2">
+      <c r="N47" t="s" s="2">
         <v>449</v>
-      </c>
-      <c r="N47" t="s" s="2">
-        <v>450</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
@@ -7877,11 +7879,11 @@
         <v>158</v>
       </c>
       <c r="Y47" t="s" s="2">
+        <v>450</v>
+      </c>
+      <c r="Z47" t="s" s="2">
         <v>451</v>
       </c>
-      <c r="Z47" t="s" s="2">
-        <v>452</v>
-      </c>
       <c r="AA47" t="s" s="2">
         <v>20</v>
       </c>
@@ -7898,7 +7900,7 @@
         <v>20</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>80</v>
@@ -7916,27 +7918,27 @@
         <v>20</v>
       </c>
       <c r="AL47" t="s" s="2">
+        <v>452</v>
+      </c>
+      <c r="AM47" t="s" s="2">
         <v>453</v>
       </c>
-      <c r="AM47" t="s" s="2">
+      <c r="AN47" t="s" s="2">
         <v>454</v>
       </c>
-      <c r="AN47" t="s" s="2">
+      <c r="AO47" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AP47" t="s" s="2">
         <v>455</v>
-      </c>
-      <c r="AO47" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AP47" t="s" s="2">
-        <v>456</v>
       </c>
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7959,19 +7961,19 @@
         <v>20</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>316</v>
+        <v>238</v>
       </c>
       <c r="L48" t="s" s="2">
+        <v>457</v>
+      </c>
+      <c r="M48" t="s" s="2">
         <v>458</v>
       </c>
-      <c r="M48" t="s" s="2">
+      <c r="N48" t="s" s="2">
         <v>459</v>
       </c>
-      <c r="N48" t="s" s="2">
+      <c r="O48" t="s" s="2">
         <v>460</v>
-      </c>
-      <c r="O48" t="s" s="2">
-        <v>461</v>
       </c>
       <c r="P48" t="s" s="2">
         <v>20</v>
@@ -7999,11 +8001,11 @@
         <v>158</v>
       </c>
       <c r="Y48" t="s" s="2">
+        <v>461</v>
+      </c>
+      <c r="Z48" t="s" s="2">
         <v>462</v>
       </c>
-      <c r="Z48" t="s" s="2">
-        <v>463</v>
-      </c>
       <c r="AA48" t="s" s="2">
         <v>20</v>
       </c>
@@ -8020,7 +8022,7 @@
         <v>20</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>80</v>
@@ -8041,10 +8043,10 @@
         <v>20</v>
       </c>
       <c r="AM48" t="s" s="2">
+        <v>463</v>
+      </c>
+      <c r="AN48" t="s" s="2">
         <v>464</v>
-      </c>
-      <c r="AN48" t="s" s="2">
-        <v>465</v>
       </c>
       <c r="AO48" t="s" s="2">
         <v>20</v>
@@ -8055,10 +8057,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -8081,16 +8083,16 @@
         <v>20</v>
       </c>
       <c r="K49" t="s" s="2">
+        <v>466</v>
+      </c>
+      <c r="L49" t="s" s="2">
         <v>467</v>
       </c>
-      <c r="L49" t="s" s="2">
+      <c r="M49" t="s" s="2">
         <v>468</v>
       </c>
-      <c r="M49" t="s" s="2">
+      <c r="N49" t="s" s="2">
         <v>469</v>
-      </c>
-      <c r="N49" t="s" s="2">
-        <v>470</v>
       </c>
       <c r="O49" s="2"/>
       <c r="P49" t="s" s="2">
@@ -8140,7 +8142,7 @@
         <v>20</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>80</v>
@@ -8158,27 +8160,27 @@
         <v>20</v>
       </c>
       <c r="AL49" t="s" s="2">
+        <v>470</v>
+      </c>
+      <c r="AM49" t="s" s="2">
         <v>471</v>
       </c>
-      <c r="AM49" t="s" s="2">
+      <c r="AN49" t="s" s="2">
         <v>472</v>
       </c>
-      <c r="AN49" t="s" s="2">
+      <c r="AO49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AP49" t="s" s="2">
         <v>473</v>
-      </c>
-      <c r="AO49" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AP49" t="s" s="2">
-        <v>474</v>
       </c>
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -8201,16 +8203,16 @@
         <v>20</v>
       </c>
       <c r="K50" t="s" s="2">
+        <v>475</v>
+      </c>
+      <c r="L50" t="s" s="2">
         <v>476</v>
       </c>
-      <c r="L50" t="s" s="2">
+      <c r="M50" t="s" s="2">
         <v>477</v>
       </c>
-      <c r="M50" t="s" s="2">
+      <c r="N50" t="s" s="2">
         <v>478</v>
-      </c>
-      <c r="N50" t="s" s="2">
-        <v>479</v>
       </c>
       <c r="O50" s="2"/>
       <c r="P50" t="s" s="2">
@@ -8260,7 +8262,7 @@
         <v>20</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>80</v>
@@ -8278,27 +8280,27 @@
         <v>20</v>
       </c>
       <c r="AL50" t="s" s="2">
+        <v>479</v>
+      </c>
+      <c r="AM50" t="s" s="2">
         <v>480</v>
       </c>
-      <c r="AM50" t="s" s="2">
+      <c r="AN50" t="s" s="2">
         <v>481</v>
       </c>
-      <c r="AN50" t="s" s="2">
+      <c r="AO50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AP50" t="s" s="2">
         <v>482</v>
-      </c>
-      <c r="AO50" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AP50" t="s" s="2">
-        <v>483</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -8321,19 +8323,19 @@
         <v>20</v>
       </c>
       <c r="K51" t="s" s="2">
+        <v>484</v>
+      </c>
+      <c r="L51" t="s" s="2">
         <v>485</v>
       </c>
-      <c r="L51" t="s" s="2">
+      <c r="M51" t="s" s="2">
         <v>486</v>
       </c>
-      <c r="M51" t="s" s="2">
+      <c r="N51" t="s" s="2">
         <v>487</v>
       </c>
-      <c r="N51" t="s" s="2">
+      <c r="O51" t="s" s="2">
         <v>488</v>
-      </c>
-      <c r="O51" t="s" s="2">
-        <v>489</v>
       </c>
       <c r="P51" t="s" s="2">
         <v>20</v>
@@ -8382,7 +8384,7 @@
         <v>20</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>80</v>
@@ -8391,22 +8393,22 @@
         <v>81</v>
       </c>
       <c r="AI51" t="s" s="2">
+        <v>489</v>
+      </c>
+      <c r="AJ51" t="s" s="2">
         <v>490</v>
       </c>
-      <c r="AJ51" t="s" s="2">
+      <c r="AK51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AL51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AM51" t="s" s="2">
         <v>491</v>
       </c>
-      <c r="AK51" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AL51" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AM51" t="s" s="2">
+      <c r="AN51" t="s" s="2">
         <v>492</v>
-      </c>
-      <c r="AN51" t="s" s="2">
-        <v>493</v>
       </c>
       <c r="AO51" t="s" s="2">
         <v>20</v>
@@ -8417,10 +8419,10 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -8535,10 +8537,10 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -8655,14 +8657,14 @@
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="E54" s="2"/>
       <c r="F54" t="s" s="2">
@@ -8684,10 +8686,10 @@
         <v>113</v>
       </c>
       <c r="L54" t="s" s="2">
+        <v>497</v>
+      </c>
+      <c r="M54" t="s" s="2">
         <v>498</v>
-      </c>
-      <c r="M54" t="s" s="2">
-        <v>499</v>
       </c>
       <c r="N54" t="s" s="2">
         <v>116</v>
@@ -8742,7 +8744,7 @@
         <v>20</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>80</v>
@@ -8777,10 +8779,10 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -8803,13 +8805,13 @@
         <v>20</v>
       </c>
       <c r="K55" t="s" s="2">
+        <v>501</v>
+      </c>
+      <c r="L55" t="s" s="2">
         <v>502</v>
       </c>
-      <c r="L55" t="s" s="2">
+      <c r="M55" t="s" s="2">
         <v>503</v>
-      </c>
-      <c r="M55" t="s" s="2">
-        <v>504</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
@@ -8860,7 +8862,7 @@
         <v>20</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>80</v>
@@ -8869,7 +8871,7 @@
         <v>92</v>
       </c>
       <c r="AI55" t="s" s="2">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="AJ55" t="s" s="2">
         <v>104</v>
@@ -8881,10 +8883,10 @@
         <v>20</v>
       </c>
       <c r="AM55" t="s" s="2">
+        <v>505</v>
+      </c>
+      <c r="AN55" t="s" s="2">
         <v>506</v>
-      </c>
-      <c r="AN55" t="s" s="2">
-        <v>507</v>
       </c>
       <c r="AO55" t="s" s="2">
         <v>20</v>
@@ -8895,10 +8897,10 @@
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -8921,13 +8923,13 @@
         <v>20</v>
       </c>
       <c r="K56" t="s" s="2">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L56" t="s" s="2">
+        <v>508</v>
+      </c>
+      <c r="M56" t="s" s="2">
         <v>509</v>
-      </c>
-      <c r="M56" t="s" s="2">
-        <v>510</v>
       </c>
       <c r="N56" s="2"/>
       <c r="O56" s="2"/>
@@ -8978,7 +8980,7 @@
         <v>20</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>80</v>
@@ -8987,7 +8989,7 @@
         <v>92</v>
       </c>
       <c r="AI56" t="s" s="2">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="AJ56" t="s" s="2">
         <v>104</v>
@@ -8999,10 +9001,10 @@
         <v>20</v>
       </c>
       <c r="AM56" t="s" s="2">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="AN56" t="s" s="2">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="AO56" t="s" s="2">
         <v>20</v>
@@ -9013,10 +9015,10 @@
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -9039,19 +9041,19 @@
         <v>20</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>316</v>
+        <v>238</v>
       </c>
       <c r="L57" t="s" s="2">
+        <v>512</v>
+      </c>
+      <c r="M57" t="s" s="2">
         <v>513</v>
       </c>
-      <c r="M57" t="s" s="2">
+      <c r="N57" t="s" s="2">
         <v>514</v>
       </c>
-      <c r="N57" t="s" s="2">
+      <c r="O57" t="s" s="2">
         <v>515</v>
-      </c>
-      <c r="O57" t="s" s="2">
-        <v>516</v>
       </c>
       <c r="P57" t="s" s="2">
         <v>20</v>
@@ -9079,11 +9081,11 @@
         <v>172</v>
       </c>
       <c r="Y57" t="s" s="2">
+        <v>516</v>
+      </c>
+      <c r="Z57" t="s" s="2">
         <v>517</v>
       </c>
-      <c r="Z57" t="s" s="2">
-        <v>518</v>
-      </c>
       <c r="AA57" t="s" s="2">
         <v>20</v>
       </c>
@@ -9100,7 +9102,7 @@
         <v>20</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>80</v>
@@ -9118,13 +9120,13 @@
         <v>20</v>
       </c>
       <c r="AL57" t="s" s="2">
+        <v>518</v>
+      </c>
+      <c r="AM57" t="s" s="2">
         <v>519</v>
       </c>
-      <c r="AM57" t="s" s="2">
-        <v>520</v>
-      </c>
       <c r="AN57" t="s" s="2">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="AO57" t="s" s="2">
         <v>20</v>
@@ -9135,10 +9137,10 @@
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -9161,19 +9163,19 @@
         <v>20</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>316</v>
+        <v>238</v>
       </c>
       <c r="L58" t="s" s="2">
+        <v>521</v>
+      </c>
+      <c r="M58" t="s" s="2">
         <v>522</v>
       </c>
-      <c r="M58" t="s" s="2">
+      <c r="N58" t="s" s="2">
         <v>523</v>
       </c>
-      <c r="N58" t="s" s="2">
+      <c r="O58" t="s" s="2">
         <v>524</v>
-      </c>
-      <c r="O58" t="s" s="2">
-        <v>525</v>
       </c>
       <c r="P58" t="s" s="2">
         <v>20</v>
@@ -9201,11 +9203,11 @@
         <v>158</v>
       </c>
       <c r="Y58" t="s" s="2">
+        <v>525</v>
+      </c>
+      <c r="Z58" t="s" s="2">
         <v>526</v>
       </c>
-      <c r="Z58" t="s" s="2">
-        <v>527</v>
-      </c>
       <c r="AA58" t="s" s="2">
         <v>20</v>
       </c>
@@ -9222,7 +9224,7 @@
         <v>20</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>80</v>
@@ -9240,13 +9242,13 @@
         <v>20</v>
       </c>
       <c r="AL58" t="s" s="2">
+        <v>518</v>
+      </c>
+      <c r="AM58" t="s" s="2">
         <v>519</v>
       </c>
-      <c r="AM58" t="s" s="2">
-        <v>520</v>
-      </c>
       <c r="AN58" t="s" s="2">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="AO58" t="s" s="2">
         <v>20</v>
@@ -9257,10 +9259,10 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -9283,17 +9285,17 @@
         <v>20</v>
       </c>
       <c r="K59" t="s" s="2">
+        <v>528</v>
+      </c>
+      <c r="L59" t="s" s="2">
         <v>529</v>
       </c>
-      <c r="L59" t="s" s="2">
+      <c r="M59" t="s" s="2">
         <v>530</v>
-      </c>
-      <c r="M59" t="s" s="2">
-        <v>531</v>
       </c>
       <c r="N59" s="2"/>
       <c r="O59" t="s" s="2">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="P59" t="s" s="2">
         <v>20</v>
@@ -9342,7 +9344,7 @@
         <v>20</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>80</v>
@@ -9366,7 +9368,7 @@
         <v>20</v>
       </c>
       <c r="AN59" t="s" s="2">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="AO59" t="s" s="2">
         <v>20</v>
@@ -9377,10 +9379,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -9406,10 +9408,10 @@
         <v>106</v>
       </c>
       <c r="L60" t="s" s="2">
+        <v>534</v>
+      </c>
+      <c r="M60" t="s" s="2">
         <v>535</v>
-      </c>
-      <c r="M60" t="s" s="2">
-        <v>536</v>
       </c>
       <c r="N60" s="2"/>
       <c r="O60" s="2"/>
@@ -9460,7 +9462,7 @@
         <v>20</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>80</v>
@@ -9481,10 +9483,10 @@
         <v>20</v>
       </c>
       <c r="AM60" t="s" s="2">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="AN60" t="s" s="2">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="AO60" t="s" s="2">
         <v>20</v>
@@ -9495,10 +9497,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -9521,16 +9523,16 @@
         <v>93</v>
       </c>
       <c r="K61" t="s" s="2">
+        <v>538</v>
+      </c>
+      <c r="L61" t="s" s="2">
         <v>539</v>
       </c>
-      <c r="L61" t="s" s="2">
+      <c r="M61" t="s" s="2">
         <v>540</v>
       </c>
-      <c r="M61" t="s" s="2">
+      <c r="N61" t="s" s="2">
         <v>541</v>
-      </c>
-      <c r="N61" t="s" s="2">
-        <v>542</v>
       </c>
       <c r="O61" s="2"/>
       <c r="P61" t="s" s="2">
@@ -9580,7 +9582,7 @@
         <v>20</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>80</v>
@@ -9601,10 +9603,10 @@
         <v>20</v>
       </c>
       <c r="AM61" t="s" s="2">
+        <v>542</v>
+      </c>
+      <c r="AN61" t="s" s="2">
         <v>543</v>
-      </c>
-      <c r="AN61" t="s" s="2">
-        <v>544</v>
       </c>
       <c r="AO61" t="s" s="2">
         <v>20</v>
@@ -9615,10 +9617,10 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -9641,16 +9643,16 @@
         <v>93</v>
       </c>
       <c r="K62" t="s" s="2">
+        <v>545</v>
+      </c>
+      <c r="L62" t="s" s="2">
         <v>546</v>
       </c>
-      <c r="L62" t="s" s="2">
+      <c r="M62" t="s" s="2">
         <v>547</v>
       </c>
-      <c r="M62" t="s" s="2">
+      <c r="N62" t="s" s="2">
         <v>548</v>
-      </c>
-      <c r="N62" t="s" s="2">
-        <v>549</v>
       </c>
       <c r="O62" s="2"/>
       <c r="P62" t="s" s="2">
@@ -9700,7 +9702,7 @@
         <v>20</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>80</v>
@@ -9721,10 +9723,10 @@
         <v>20</v>
       </c>
       <c r="AM62" t="s" s="2">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="AN62" t="s" s="2">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="AO62" t="s" s="2">
         <v>20</v>
@@ -9735,10 +9737,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -9761,19 +9763,19 @@
         <v>93</v>
       </c>
       <c r="K63" t="s" s="2">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="L63" t="s" s="2">
+        <v>551</v>
+      </c>
+      <c r="M63" t="s" s="2">
         <v>552</v>
       </c>
-      <c r="M63" t="s" s="2">
+      <c r="N63" t="s" s="2">
         <v>553</v>
       </c>
-      <c r="N63" t="s" s="2">
+      <c r="O63" t="s" s="2">
         <v>554</v>
-      </c>
-      <c r="O63" t="s" s="2">
-        <v>555</v>
       </c>
       <c r="P63" t="s" s="2">
         <v>20</v>
@@ -9822,7 +9824,7 @@
         <v>20</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>80</v>
@@ -9843,10 +9845,10 @@
         <v>20</v>
       </c>
       <c r="AM63" t="s" s="2">
+        <v>555</v>
+      </c>
+      <c r="AN63" t="s" s="2">
         <v>556</v>
-      </c>
-      <c r="AN63" t="s" s="2">
-        <v>557</v>
       </c>
       <c r="AO63" t="s" s="2">
         <v>20</v>
@@ -9857,10 +9859,10 @@
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -9975,10 +9977,10 @@
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -10095,14 +10097,14 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="E66" s="2"/>
       <c r="F66" t="s" s="2">
@@ -10124,10 +10126,10 @@
         <v>113</v>
       </c>
       <c r="L66" t="s" s="2">
+        <v>497</v>
+      </c>
+      <c r="M66" t="s" s="2">
         <v>498</v>
-      </c>
-      <c r="M66" t="s" s="2">
-        <v>499</v>
       </c>
       <c r="N66" t="s" s="2">
         <v>116</v>
@@ -10182,7 +10184,7 @@
         <v>20</v>
       </c>
       <c r="AF66" t="s" s="2">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="AG66" t="s" s="2">
         <v>80</v>
@@ -10217,10 +10219,10 @@
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -10243,19 +10245,19 @@
         <v>93</v>
       </c>
       <c r="K67" t="s" s="2">
-        <v>316</v>
+        <v>238</v>
       </c>
       <c r="L67" t="s" s="2">
+        <v>561</v>
+      </c>
+      <c r="M67" t="s" s="2">
         <v>562</v>
       </c>
-      <c r="M67" t="s" s="2">
+      <c r="N67" t="s" s="2">
         <v>563</v>
       </c>
-      <c r="N67" t="s" s="2">
-        <v>564</v>
-      </c>
       <c r="O67" t="s" s="2">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="P67" t="s" s="2">
         <v>20</v>
@@ -10283,11 +10285,11 @@
         <v>158</v>
       </c>
       <c r="Y67" t="s" s="2">
+        <v>564</v>
+      </c>
+      <c r="Z67" t="s" s="2">
         <v>565</v>
       </c>
-      <c r="Z67" t="s" s="2">
-        <v>566</v>
-      </c>
       <c r="AA67" t="s" s="2">
         <v>20</v>
       </c>
@@ -10304,7 +10306,7 @@
         <v>20</v>
       </c>
       <c r="AF67" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="AG67" t="s" s="2">
         <v>92</v>
@@ -10322,16 +10324,16 @@
         <v>20</v>
       </c>
       <c r="AL67" t="s" s="2">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="AM67" t="s" s="2">
+        <v>343</v>
+      </c>
+      <c r="AN67" t="s" s="2">
+        <v>344</v>
+      </c>
+      <c r="AO67" t="s" s="2">
         <v>345</v>
-      </c>
-      <c r="AN67" t="s" s="2">
-        <v>346</v>
-      </c>
-      <c r="AO67" t="s" s="2">
-        <v>347</v>
       </c>
       <c r="AP67" t="s" s="2">
         <v>20</v>
@@ -10339,10 +10341,10 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -10365,19 +10367,19 @@
         <v>93</v>
       </c>
       <c r="K68" t="s" s="2">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="L68" t="s" s="2">
+        <v>568</v>
+      </c>
+      <c r="M68" t="s" s="2">
         <v>569</v>
       </c>
-      <c r="M68" t="s" s="2">
+      <c r="N68" t="s" s="2">
         <v>570</v>
       </c>
-      <c r="N68" t="s" s="2">
-        <v>571</v>
-      </c>
       <c r="O68" t="s" s="2">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="P68" t="s" s="2">
         <v>20</v>
@@ -10426,7 +10428,7 @@
         <v>20</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>80</v>
@@ -10444,27 +10446,27 @@
         <v>20</v>
       </c>
       <c r="AL68" t="s" s="2">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="AM68" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="AN68" t="s" s="2">
+        <v>414</v>
+      </c>
+      <c r="AO68" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AP68" t="s" s="2">
         <v>415</v>
-      </c>
-      <c r="AN68" t="s" s="2">
-        <v>416</v>
-      </c>
-      <c r="AO68" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AP68" t="s" s="2">
-        <v>417</v>
       </c>
     </row>
     <row r="69" hidden="true">
       <c r="A69" t="s" s="2">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -10487,19 +10489,19 @@
         <v>20</v>
       </c>
       <c r="K69" t="s" s="2">
-        <v>239</v>
+        <v>417</v>
       </c>
       <c r="L69" t="s" s="2">
+        <v>573</v>
+      </c>
+      <c r="M69" t="s" s="2">
         <v>574</v>
       </c>
-      <c r="M69" t="s" s="2">
+      <c r="N69" t="s" s="2">
         <v>575</v>
       </c>
-      <c r="N69" t="s" s="2">
-        <v>576</v>
-      </c>
       <c r="O69" t="s" s="2">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="P69" t="s" s="2">
         <v>20</v>
@@ -10527,11 +10529,11 @@
         <v>150</v>
       </c>
       <c r="Y69" t="s" s="2">
+        <v>422</v>
+      </c>
+      <c r="Z69" t="s" s="2">
         <v>423</v>
       </c>
-      <c r="Z69" t="s" s="2">
-        <v>424</v>
-      </c>
       <c r="AA69" t="s" s="2">
         <v>20</v>
       </c>
@@ -10548,7 +10550,7 @@
         <v>20</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>80</v>
@@ -10557,7 +10559,7 @@
         <v>92</v>
       </c>
       <c r="AI69" t="s" s="2">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="AJ69" t="s" s="2">
         <v>104</v>
@@ -10572,7 +10574,7 @@
         <v>191</v>
       </c>
       <c r="AN69" t="s" s="2">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="AO69" t="s" s="2">
         <v>20</v>
@@ -10583,14 +10585,14 @@
     </row>
     <row r="70" hidden="true">
       <c r="A70" t="s" s="2">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E70" s="2"/>
       <c r="F70" t="s" s="2">
@@ -10609,19 +10611,19 @@
         <v>20</v>
       </c>
       <c r="K70" t="s" s="2">
-        <v>316</v>
+        <v>238</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="M70" t="s" s="2">
+        <v>429</v>
+      </c>
+      <c r="N70" t="s" s="2">
         <v>430</v>
       </c>
-      <c r="N70" t="s" s="2">
+      <c r="O70" t="s" s="2">
         <v>431</v>
-      </c>
-      <c r="O70" t="s" s="2">
-        <v>432</v>
       </c>
       <c r="P70" t="s" s="2">
         <v>20</v>
@@ -10649,11 +10651,11 @@
         <v>150</v>
       </c>
       <c r="Y70" t="s" s="2">
+        <v>432</v>
+      </c>
+      <c r="Z70" t="s" s="2">
         <v>433</v>
       </c>
-      <c r="Z70" t="s" s="2">
-        <v>434</v>
-      </c>
       <c r="AA70" t="s" s="2">
         <v>20</v>
       </c>
@@ -10670,7 +10672,7 @@
         <v>20</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>80</v>
@@ -10688,27 +10690,27 @@
         <v>20</v>
       </c>
       <c r="AL70" t="s" s="2">
+        <v>434</v>
+      </c>
+      <c r="AM70" t="s" s="2">
         <v>435</v>
       </c>
-      <c r="AM70" t="s" s="2">
+      <c r="AN70" t="s" s="2">
         <v>436</v>
       </c>
-      <c r="AN70" t="s" s="2">
+      <c r="AO70" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AP70" t="s" s="2">
         <v>437</v>
-      </c>
-      <c r="AO70" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AP70" t="s" s="2">
-        <v>438</v>
       </c>
     </row>
     <row r="71" hidden="true">
       <c r="A71" t="s" s="2">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -10731,19 +10733,19 @@
         <v>20</v>
       </c>
       <c r="K71" t="s" s="2">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="L71" t="s" s="2">
+        <v>580</v>
+      </c>
+      <c r="M71" t="s" s="2">
         <v>581</v>
       </c>
-      <c r="M71" t="s" s="2">
+      <c r="N71" t="s" s="2">
         <v>582</v>
       </c>
-      <c r="N71" t="s" s="2">
-        <v>583</v>
-      </c>
       <c r="O71" t="s" s="2">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="P71" t="s" s="2">
         <v>20</v>
@@ -10792,7 +10794,7 @@
         <v>20</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>80</v>
@@ -10813,10 +10815,10 @@
         <v>20</v>
       </c>
       <c r="AM71" t="s" s="2">
+        <v>491</v>
+      </c>
+      <c r="AN71" t="s" s="2">
         <v>492</v>
-      </c>
-      <c r="AN71" t="s" s="2">
-        <v>493</v>
       </c>
       <c r="AO71" t="s" s="2">
         <v>20</v>
@@ -10827,10 +10829,10 @@
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -10945,10 +10947,10 @@
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -11065,14 +11067,14 @@
     </row>
     <row r="74" hidden="true">
       <c r="A74" t="s" s="2">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="E74" s="2"/>
       <c r="F74" t="s" s="2">
@@ -11094,10 +11096,10 @@
         <v>113</v>
       </c>
       <c r="L74" t="s" s="2">
+        <v>497</v>
+      </c>
+      <c r="M74" t="s" s="2">
         <v>498</v>
-      </c>
-      <c r="M74" t="s" s="2">
-        <v>499</v>
       </c>
       <c r="N74" t="s" s="2">
         <v>116</v>
@@ -11152,7 +11154,7 @@
         <v>20</v>
       </c>
       <c r="AF74" t="s" s="2">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="AG74" t="s" s="2">
         <v>80</v>
@@ -11187,10 +11189,10 @@
     </row>
     <row r="75" hidden="true">
       <c r="A75" t="s" s="2">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -11213,13 +11215,13 @@
         <v>20</v>
       </c>
       <c r="K75" t="s" s="2">
+        <v>501</v>
+      </c>
+      <c r="L75" t="s" s="2">
         <v>502</v>
       </c>
-      <c r="L75" t="s" s="2">
+      <c r="M75" t="s" s="2">
         <v>503</v>
-      </c>
-      <c r="M75" t="s" s="2">
-        <v>504</v>
       </c>
       <c r="N75" s="2"/>
       <c r="O75" s="2"/>
@@ -11270,7 +11272,7 @@
         <v>20</v>
       </c>
       <c r="AF75" t="s" s="2">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="AG75" t="s" s="2">
         <v>80</v>
@@ -11279,7 +11281,7 @@
         <v>92</v>
       </c>
       <c r="AI75" t="s" s="2">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="AJ75" t="s" s="2">
         <v>104</v>
@@ -11291,10 +11293,10 @@
         <v>20</v>
       </c>
       <c r="AM75" t="s" s="2">
+        <v>505</v>
+      </c>
+      <c r="AN75" t="s" s="2">
         <v>506</v>
-      </c>
-      <c r="AN75" t="s" s="2">
-        <v>507</v>
       </c>
       <c r="AO75" t="s" s="2">
         <v>20</v>
@@ -11305,10 +11307,10 @@
     </row>
     <row r="76" hidden="true">
       <c r="A76" t="s" s="2">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -11331,13 +11333,13 @@
         <v>20</v>
       </c>
       <c r="K76" t="s" s="2">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L76" t="s" s="2">
+        <v>508</v>
+      </c>
+      <c r="M76" t="s" s="2">
         <v>509</v>
-      </c>
-      <c r="M76" t="s" s="2">
-        <v>510</v>
       </c>
       <c r="N76" s="2"/>
       <c r="O76" s="2"/>
@@ -11388,7 +11390,7 @@
         <v>20</v>
       </c>
       <c r="AF76" t="s" s="2">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>80</v>
@@ -11397,7 +11399,7 @@
         <v>92</v>
       </c>
       <c r="AI76" t="s" s="2">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="AJ76" t="s" s="2">
         <v>104</v>
@@ -11409,10 +11411,10 @@
         <v>20</v>
       </c>
       <c r="AM76" t="s" s="2">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="AN76" t="s" s="2">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="AO76" t="s" s="2">
         <v>20</v>
@@ -11423,10 +11425,10 @@
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -11449,19 +11451,19 @@
         <v>20</v>
       </c>
       <c r="K77" t="s" s="2">
-        <v>316</v>
+        <v>238</v>
       </c>
       <c r="L77" t="s" s="2">
+        <v>512</v>
+      </c>
+      <c r="M77" t="s" s="2">
         <v>513</v>
       </c>
-      <c r="M77" t="s" s="2">
+      <c r="N77" t="s" s="2">
         <v>514</v>
       </c>
-      <c r="N77" t="s" s="2">
+      <c r="O77" t="s" s="2">
         <v>515</v>
-      </c>
-      <c r="O77" t="s" s="2">
-        <v>516</v>
       </c>
       <c r="P77" t="s" s="2">
         <v>20</v>
@@ -11489,10 +11491,10 @@
         <v>172</v>
       </c>
       <c r="Y77" t="s" s="2">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="Z77" t="s" s="2">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="AA77" t="s" s="2">
         <v>20</v>
@@ -11510,7 +11512,7 @@
         <v>20</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>80</v>
@@ -11528,13 +11530,13 @@
         <v>20</v>
       </c>
       <c r="AL77" t="s" s="2">
+        <v>518</v>
+      </c>
+      <c r="AM77" t="s" s="2">
         <v>519</v>
       </c>
-      <c r="AM77" t="s" s="2">
-        <v>520</v>
-      </c>
       <c r="AN77" t="s" s="2">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="AO77" t="s" s="2">
         <v>20</v>
@@ -11545,10 +11547,10 @@
     </row>
     <row r="78" hidden="true">
       <c r="A78" t="s" s="2">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -11571,19 +11573,19 @@
         <v>20</v>
       </c>
       <c r="K78" t="s" s="2">
-        <v>316</v>
+        <v>238</v>
       </c>
       <c r="L78" t="s" s="2">
+        <v>521</v>
+      </c>
+      <c r="M78" t="s" s="2">
         <v>522</v>
       </c>
-      <c r="M78" t="s" s="2">
+      <c r="N78" t="s" s="2">
         <v>523</v>
       </c>
-      <c r="N78" t="s" s="2">
+      <c r="O78" t="s" s="2">
         <v>524</v>
-      </c>
-      <c r="O78" t="s" s="2">
-        <v>525</v>
       </c>
       <c r="P78" t="s" s="2">
         <v>20</v>
@@ -11611,10 +11613,10 @@
         <v>158</v>
       </c>
       <c r="Y78" t="s" s="2">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="Z78" t="s" s="2">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="AA78" t="s" s="2">
         <v>20</v>
@@ -11632,7 +11634,7 @@
         <v>20</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>80</v>
@@ -11650,13 +11652,13 @@
         <v>20</v>
       </c>
       <c r="AL78" t="s" s="2">
+        <v>518</v>
+      </c>
+      <c r="AM78" t="s" s="2">
         <v>519</v>
       </c>
-      <c r="AM78" t="s" s="2">
-        <v>520</v>
-      </c>
       <c r="AN78" t="s" s="2">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="AO78" t="s" s="2">
         <v>20</v>
@@ -11667,10 +11669,10 @@
     </row>
     <row r="79" hidden="true">
       <c r="A79" t="s" s="2">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -11693,17 +11695,17 @@
         <v>20</v>
       </c>
       <c r="K79" t="s" s="2">
+        <v>528</v>
+      </c>
+      <c r="L79" t="s" s="2">
         <v>529</v>
       </c>
-      <c r="L79" t="s" s="2">
+      <c r="M79" t="s" s="2">
         <v>530</v>
-      </c>
-      <c r="M79" t="s" s="2">
-        <v>531</v>
       </c>
       <c r="N79" s="2"/>
       <c r="O79" t="s" s="2">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="P79" t="s" s="2">
         <v>20</v>
@@ -11752,7 +11754,7 @@
         <v>20</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>80</v>
@@ -11776,7 +11778,7 @@
         <v>20</v>
       </c>
       <c r="AN79" t="s" s="2">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="AO79" t="s" s="2">
         <v>20</v>
@@ -11787,10 +11789,10 @@
     </row>
     <row r="80" hidden="true">
       <c r="A80" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -11816,10 +11818,10 @@
         <v>106</v>
       </c>
       <c r="L80" t="s" s="2">
+        <v>534</v>
+      </c>
+      <c r="M80" t="s" s="2">
         <v>535</v>
-      </c>
-      <c r="M80" t="s" s="2">
-        <v>536</v>
       </c>
       <c r="N80" s="2"/>
       <c r="O80" s="2"/>
@@ -11870,7 +11872,7 @@
         <v>20</v>
       </c>
       <c r="AF80" t="s" s="2">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="AG80" t="s" s="2">
         <v>80</v>
@@ -11891,10 +11893,10 @@
         <v>20</v>
       </c>
       <c r="AM80" t="s" s="2">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="AN80" t="s" s="2">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="AO80" t="s" s="2">
         <v>20</v>

</xml_diff>